<commit_message>
Keep the generator independent of the holidays package
Silent anomalies avoided public holidays through the holidays package, so
the ledger, and with it the fixtures, changed with the package version
(CI has a newer calendar). They now fall on any weekday; one on a public
holiday is a chance hit, like Benford. Fixtures rebuilt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fixtures/idea_exports/Benford Starting 4.xlsx
+++ b/fixtures/idea_exports/Benford Starting 4.xlsx
@@ -24990,7 +24990,7 @@
     </row>
     <row r="723">
       <c r="A723" t="n">
-        <v>6065</v>
+        <v>6066</v>
       </c>
       <c r="B723" s="2" t="n">
         <v>45771</v>
@@ -25024,7 +25024,7 @@
     </row>
     <row r="724">
       <c r="A724" t="n">
-        <v>6084</v>
+        <v>6085</v>
       </c>
       <c r="B724" s="2" t="n">
         <v>45771</v>
@@ -25058,7 +25058,7 @@
     </row>
     <row r="725">
       <c r="A725" t="n">
-        <v>6092</v>
+        <v>6093</v>
       </c>
       <c r="B725" s="2" t="n">
         <v>45771</v>
@@ -25092,7 +25092,7 @@
     </row>
     <row r="726">
       <c r="A726" t="n">
-        <v>6093</v>
+        <v>6094</v>
       </c>
       <c r="B726" s="2" t="n">
         <v>45771</v>
@@ -25126,7 +25126,7 @@
     </row>
     <row r="727">
       <c r="A727" t="n">
-        <v>6100</v>
+        <v>6101</v>
       </c>
       <c r="B727" s="2" t="n">
         <v>45771</v>
@@ -25160,7 +25160,7 @@
     </row>
     <row r="728">
       <c r="A728" t="n">
-        <v>6118</v>
+        <v>6119</v>
       </c>
       <c r="B728" s="2" t="n">
         <v>45771</v>
@@ -25194,7 +25194,7 @@
     </row>
     <row r="729">
       <c r="A729" t="n">
-        <v>6120</v>
+        <v>6121</v>
       </c>
       <c r="B729" s="2" t="n">
         <v>45772</v>
@@ -42194,7 +42194,7 @@
     </row>
     <row r="1229">
       <c r="A1229" t="n">
-        <v>10329</v>
+        <v>10330</v>
       </c>
       <c r="B1229" s="2" t="n">
         <v>45847</v>
@@ -42228,7 +42228,7 @@
     </row>
     <row r="1230">
       <c r="A1230" t="n">
-        <v>10337</v>
+        <v>10338</v>
       </c>
       <c r="B1230" s="2" t="n">
         <v>45847</v>
@@ -42262,7 +42262,7 @@
     </row>
     <row r="1231">
       <c r="A1231" t="n">
-        <v>10342</v>
+        <v>10343</v>
       </c>
       <c r="B1231" s="2" t="n">
         <v>45847</v>
@@ -42296,7 +42296,7 @@
     </row>
     <row r="1232">
       <c r="A1232" t="n">
-        <v>10346</v>
+        <v>10347</v>
       </c>
       <c r="B1232" s="2" t="n">
         <v>45847</v>
@@ -42330,7 +42330,7 @@
     </row>
     <row r="1233">
       <c r="A1233" t="n">
-        <v>10352</v>
+        <v>10353</v>
       </c>
       <c r="B1233" s="2" t="n">
         <v>45847</v>
@@ -42364,7 +42364,7 @@
     </row>
     <row r="1234">
       <c r="A1234" t="n">
-        <v>10354</v>
+        <v>10355</v>
       </c>
       <c r="B1234" s="2" t="n">
         <v>45847</v>
@@ -42398,7 +42398,7 @@
     </row>
     <row r="1235">
       <c r="A1235" t="n">
-        <v>10366</v>
+        <v>10367</v>
       </c>
       <c r="B1235" s="2" t="n">
         <v>45848</v>
@@ -42432,7 +42432,7 @@
     </row>
     <row r="1236">
       <c r="A1236" t="n">
-        <v>10368</v>
+        <v>10369</v>
       </c>
       <c r="B1236" s="2" t="n">
         <v>45848</v>
@@ -42466,7 +42466,7 @@
     </row>
     <row r="1237">
       <c r="A1237" t="n">
-        <v>10369</v>
+        <v>10370</v>
       </c>
       <c r="B1237" s="2" t="n">
         <v>45848</v>
@@ -42500,7 +42500,7 @@
     </row>
     <row r="1238">
       <c r="A1238" t="n">
-        <v>10376</v>
+        <v>10377</v>
       </c>
       <c r="B1238" s="2" t="n">
         <v>45848</v>
@@ -42534,7 +42534,7 @@
     </row>
     <row r="1239">
       <c r="A1239" t="n">
-        <v>10386</v>
+        <v>10387</v>
       </c>
       <c r="B1239" s="2" t="n">
         <v>45848</v>
@@ -42568,7 +42568,7 @@
     </row>
     <row r="1240">
       <c r="A1240" t="n">
-        <v>10396</v>
+        <v>10397</v>
       </c>
       <c r="B1240" s="2" t="n">
         <v>45848</v>
@@ -42602,7 +42602,7 @@
     </row>
     <row r="1241">
       <c r="A1241" t="n">
-        <v>10405</v>
+        <v>10406</v>
       </c>
       <c r="B1241" s="2" t="n">
         <v>45848</v>
@@ -42636,7 +42636,7 @@
     </row>
     <row r="1242">
       <c r="A1242" t="n">
-        <v>10406</v>
+        <v>10407</v>
       </c>
       <c r="B1242" s="2" t="n">
         <v>45848</v>
@@ -42670,7 +42670,7 @@
     </row>
     <row r="1243">
       <c r="A1243" t="n">
-        <v>10418</v>
+        <v>10419</v>
       </c>
       <c r="B1243" s="2" t="n">
         <v>45848</v>
@@ -42704,7 +42704,7 @@
     </row>
     <row r="1244">
       <c r="A1244" t="n">
-        <v>10421</v>
+        <v>10422</v>
       </c>
       <c r="B1244" s="2" t="n">
         <v>45848</v>
@@ -42738,7 +42738,7 @@
     </row>
     <row r="1245">
       <c r="A1245" t="n">
-        <v>10441</v>
+        <v>10442</v>
       </c>
       <c r="B1245" s="2" t="n">
         <v>45849</v>
@@ -42772,7 +42772,7 @@
     </row>
     <row r="1246">
       <c r="A1246" t="n">
-        <v>10451</v>
+        <v>10452</v>
       </c>
       <c r="B1246" s="2" t="n">
         <v>45849</v>
@@ -42806,7 +42806,7 @@
     </row>
     <row r="1247">
       <c r="A1247" t="n">
-        <v>10454</v>
+        <v>10455</v>
       </c>
       <c r="B1247" s="2" t="n">
         <v>45849</v>
@@ -50150,7 +50150,7 @@
     </row>
     <row r="1463">
       <c r="A1463" t="n">
-        <v>12189</v>
+        <v>12190</v>
       </c>
       <c r="B1463" s="2" t="n">
         <v>45881</v>
@@ -50184,7 +50184,7 @@
     </row>
     <row r="1464">
       <c r="A1464" t="n">
-        <v>12191</v>
+        <v>12192</v>
       </c>
       <c r="B1464" s="2" t="n">
         <v>45881</v>
@@ -50218,7 +50218,7 @@
     </row>
     <row r="1465">
       <c r="A1465" t="n">
-        <v>12200</v>
+        <v>12201</v>
       </c>
       <c r="B1465" s="2" t="n">
         <v>45881</v>
@@ -50252,7 +50252,7 @@
     </row>
     <row r="1466">
       <c r="A1466" t="n">
-        <v>12206</v>
+        <v>12207</v>
       </c>
       <c r="B1466" s="2" t="n">
         <v>45881</v>
@@ -50286,7 +50286,7 @@
     </row>
     <row r="1467">
       <c r="A1467" t="n">
-        <v>12209</v>
+        <v>12210</v>
       </c>
       <c r="B1467" s="2" t="n">
         <v>45881</v>
@@ -50320,7 +50320,7 @@
     </row>
     <row r="1468">
       <c r="A1468" t="n">
-        <v>12216</v>
+        <v>12217</v>
       </c>
       <c r="B1468" s="2" t="n">
         <v>45881</v>
@@ -50354,7 +50354,7 @@
     </row>
     <row r="1469">
       <c r="A1469" t="n">
-        <v>12224</v>
+        <v>12225</v>
       </c>
       <c r="B1469" s="2" t="n">
         <v>45882</v>
@@ -50388,7 +50388,7 @@
     </row>
     <row r="1470">
       <c r="A1470" t="n">
-        <v>12231</v>
+        <v>12232</v>
       </c>
       <c r="B1470" s="2" t="n">
         <v>45882</v>
@@ -50422,7 +50422,7 @@
     </row>
     <row r="1471">
       <c r="A1471" t="n">
-        <v>12244</v>
+        <v>12245</v>
       </c>
       <c r="B1471" s="2" t="n">
         <v>45882</v>
@@ -50456,7 +50456,7 @@
     </row>
     <row r="1472">
       <c r="A1472" t="n">
-        <v>12246</v>
+        <v>12247</v>
       </c>
       <c r="B1472" s="2" t="n">
         <v>45882</v>
@@ -50490,7 +50490,7 @@
     </row>
     <row r="1473">
       <c r="A1473" t="n">
-        <v>12251</v>
+        <v>12252</v>
       </c>
       <c r="B1473" s="2" t="n">
         <v>45882</v>
@@ -50524,7 +50524,7 @@
     </row>
     <row r="1474">
       <c r="A1474" t="n">
-        <v>12258</v>
+        <v>12259</v>
       </c>
       <c r="B1474" s="2" t="n">
         <v>45882</v>
@@ -68238,7 +68238,7 @@
     </row>
     <row r="1995">
       <c r="A1995" t="n">
-        <v>16725</v>
+        <v>16724</v>
       </c>
       <c r="B1995" s="2" t="n">
         <v>45961</v>
@@ -68272,7 +68272,7 @@
     </row>
     <row r="1996">
       <c r="A1996" t="n">
-        <v>16730</v>
+        <v>16729</v>
       </c>
       <c r="B1996" s="2" t="n">
         <v>45961</v>
@@ -68306,7 +68306,7 @@
     </row>
     <row r="1997">
       <c r="A1997" t="n">
-        <v>16741</v>
+        <v>16740</v>
       </c>
       <c r="B1997" s="2" t="n">
         <v>45961</v>
@@ -68340,7 +68340,7 @@
     </row>
     <row r="1998">
       <c r="A1998" t="n">
-        <v>16750</v>
+        <v>16749</v>
       </c>
       <c r="B1998" s="2" t="n">
         <v>45961</v>
@@ -68374,7 +68374,7 @@
     </row>
     <row r="1999">
       <c r="A1999" t="n">
-        <v>16755</v>
+        <v>16754</v>
       </c>
       <c r="B1999" s="2" t="n">
         <v>45961</v>
@@ -68408,7 +68408,7 @@
     </row>
     <row r="2000">
       <c r="A2000" t="n">
-        <v>16781</v>
+        <v>16780</v>
       </c>
       <c r="B2000" s="2" t="n">
         <v>45964</v>
@@ -68442,7 +68442,7 @@
     </row>
     <row r="2001">
       <c r="A2001" t="n">
-        <v>16783</v>
+        <v>16782</v>
       </c>
       <c r="B2001" s="2" t="n">
         <v>45964</v>
@@ -72522,7 +72522,7 @@
     </row>
     <row r="2121">
       <c r="A2121" t="n">
-        <v>17527</v>
+        <v>17526</v>
       </c>
       <c r="B2121" s="2" t="n">
         <v>45975</v>
@@ -72556,7 +72556,7 @@
     </row>
     <row r="2122">
       <c r="A2122" t="n">
-        <v>17547</v>
+        <v>17545</v>
       </c>
       <c r="B2122" s="2" t="n">
         <v>45975</v>
@@ -72590,7 +72590,7 @@
     </row>
     <row r="2123">
       <c r="A2123" t="n">
-        <v>17555</v>
+        <v>17553</v>
       </c>
       <c r="B2123" s="2" t="n">
         <v>45975</v>
@@ -72624,7 +72624,7 @@
     </row>
     <row r="2124">
       <c r="A2124" t="n">
-        <v>17560</v>
+        <v>17558</v>
       </c>
       <c r="B2124" s="2" t="n">
         <v>45975</v>
@@ -72658,7 +72658,7 @@
     </row>
     <row r="2125">
       <c r="A2125" t="n">
-        <v>17564</v>
+        <v>17562</v>
       </c>
       <c r="B2125" s="2" t="n">
         <v>45975</v>
@@ -72692,7 +72692,7 @@
     </row>
     <row r="2126">
       <c r="A2126" t="n">
-        <v>17565</v>
+        <v>17563</v>
       </c>
       <c r="B2126" s="2" t="n">
         <v>45975</v>
@@ -72726,7 +72726,7 @@
     </row>
     <row r="2127">
       <c r="A2127" t="n">
-        <v>17566</v>
+        <v>17564</v>
       </c>
       <c r="B2127" s="2" t="n">
         <v>45975</v>
@@ -72760,7 +72760,7 @@
     </row>
     <row r="2128">
       <c r="A2128" t="n">
-        <v>17570</v>
+        <v>17568</v>
       </c>
       <c r="B2128" s="2" t="n">
         <v>45975</v>
@@ -72794,7 +72794,7 @@
     </row>
     <row r="2129">
       <c r="A2129" t="n">
-        <v>17572</v>
+        <v>17570</v>
       </c>
       <c r="B2129" s="2" t="n">
         <v>45975</v>
@@ -72828,7 +72828,7 @@
     </row>
     <row r="2130">
       <c r="A2130" t="n">
-        <v>17576</v>
+        <v>17574</v>
       </c>
       <c r="B2130" s="2" t="n">
         <v>45976</v>
@@ -72862,7 +72862,7 @@
     </row>
     <row r="2131">
       <c r="A2131" t="n">
-        <v>17580</v>
+        <v>17578</v>
       </c>
       <c r="B2131" s="2" t="n">
         <v>45977</v>
@@ -72896,7 +72896,7 @@
     </row>
     <row r="2132">
       <c r="A2132" t="n">
-        <v>17586</v>
+        <v>17584</v>
       </c>
       <c r="B2132" s="2" t="n">
         <v>45978</v>
@@ -72930,7 +72930,7 @@
     </row>
     <row r="2133">
       <c r="A2133" t="n">
-        <v>17588</v>
+        <v>17586</v>
       </c>
       <c r="B2133" s="2" t="n">
         <v>45978</v>
@@ -75004,58 +75004,58 @@
     </row>
     <row r="2194">
       <c r="A2194" t="n">
-        <v>18127</v>
+        <v>18137</v>
       </c>
       <c r="B2194" s="2" t="n">
         <v>45987</v>
       </c>
       <c r="C2194" t="inlineStr">
         <is>
-          <t>VAT Payable</t>
+          <t>Accounts Payable</t>
         </is>
       </c>
       <c r="D2194" t="inlineStr">
         <is>
-          <t>Accrual</t>
+          <t>Purchase invoice</t>
         </is>
       </c>
       <c r="E2194" t="inlineStr">
         <is>
-          <t>user_c</t>
+          <t>user_b</t>
         </is>
       </c>
       <c r="F2194" t="inlineStr">
         <is>
-          <t>manager_2</t>
+          <t>manager_1</t>
         </is>
       </c>
       <c r="G2194" t="n">
-        <v>48959.3</v>
+        <v>0</v>
       </c>
       <c r="H2194" t="n">
-        <v>0</v>
+        <v>497.08</v>
       </c>
     </row>
     <row r="2195">
       <c r="A2195" t="n">
-        <v>18138</v>
+        <v>18144</v>
       </c>
       <c r="B2195" s="2" t="n">
         <v>45987</v>
       </c>
       <c r="C2195" t="inlineStr">
         <is>
-          <t>Accounts Payable</t>
+          <t>Cost of Sales</t>
         </is>
       </c>
       <c r="D2195" t="inlineStr">
         <is>
-          <t>Purchase invoice</t>
+          <t>Customer receipt</t>
         </is>
       </c>
       <c r="E2195" t="inlineStr">
         <is>
-          <t>user_b</t>
+          <t>user_d</t>
         </is>
       </c>
       <c r="F2195" t="inlineStr">
@@ -75064,10 +75064,10 @@
         </is>
       </c>
       <c r="G2195" t="n">
-        <v>0</v>
+        <v>402.42</v>
       </c>
       <c r="H2195" t="n">
-        <v>497.08</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2196">
@@ -75079,26 +75079,26 @@
       </c>
       <c r="C2196" t="inlineStr">
         <is>
-          <t>Cost of Sales</t>
+          <t>Accounts Receivable</t>
         </is>
       </c>
       <c r="D2196" t="inlineStr">
         <is>
-          <t>Customer receipt</t>
+          <t>Staff travel claim</t>
         </is>
       </c>
       <c r="E2196" t="inlineStr">
         <is>
-          <t>user_d</t>
+          <t>user_c</t>
         </is>
       </c>
       <c r="F2196" t="inlineStr">
         <is>
-          <t>manager_1</t>
+          <t>manager_2</t>
         </is>
       </c>
       <c r="G2196" t="n">
-        <v>402.42</v>
+        <v>424.83</v>
       </c>
       <c r="H2196" t="n">
         <v>0</v>
@@ -75106,33 +75106,33 @@
     </row>
     <row r="2197">
       <c r="A2197" t="n">
-        <v>18146</v>
+        <v>18156</v>
       </c>
       <c r="B2197" s="2" t="n">
-        <v>45987</v>
+        <v>45988</v>
       </c>
       <c r="C2197" t="inlineStr">
         <is>
-          <t>Accounts Receivable</t>
+          <t>Accounts Payable</t>
         </is>
       </c>
       <c r="D2197" t="inlineStr">
         <is>
-          <t>Staff travel claim</t>
+          <t>Utility bill</t>
         </is>
       </c>
       <c r="E2197" t="inlineStr">
         <is>
-          <t>user_c</t>
+          <t>user_a</t>
         </is>
       </c>
       <c r="F2197" t="inlineStr">
         <is>
-          <t>manager_2</t>
+          <t>manager_1</t>
         </is>
       </c>
       <c r="G2197" t="n">
-        <v>424.83</v>
+        <v>463.9</v>
       </c>
       <c r="H2197" t="n">
         <v>0</v>
@@ -75147,17 +75147,17 @@
       </c>
       <c r="C2198" t="inlineStr">
         <is>
-          <t>Accounts Payable</t>
+          <t>Cash at Bank</t>
         </is>
       </c>
       <c r="D2198" t="inlineStr">
         <is>
-          <t>Utility bill</t>
+          <t>Staff travel claim</t>
         </is>
       </c>
       <c r="E2198" t="inlineStr">
         <is>
-          <t>user_a</t>
+          <t>user_e</t>
         </is>
       </c>
       <c r="F2198" t="inlineStr">
@@ -75166,7 +75166,7 @@
         </is>
       </c>
       <c r="G2198" t="n">
-        <v>463.9</v>
+        <v>436.49</v>
       </c>
       <c r="H2198" t="n">
         <v>0</v>
@@ -75174,19 +75174,19 @@
     </row>
     <row r="2199">
       <c r="A2199" t="n">
-        <v>18158</v>
+        <v>18161</v>
       </c>
       <c r="B2199" s="2" t="n">
         <v>45988</v>
       </c>
       <c r="C2199" t="inlineStr">
         <is>
-          <t>Cash at Bank</t>
+          <t>Accounts Receivable</t>
         </is>
       </c>
       <c r="D2199" t="inlineStr">
         <is>
-          <t>Staff travel claim</t>
+          <t>Customer receipt</t>
         </is>
       </c>
       <c r="E2199" t="inlineStr">
@@ -75196,11 +75196,11 @@
       </c>
       <c r="F2199" t="inlineStr">
         <is>
-          <t>manager_1</t>
+          <t>manager_2</t>
         </is>
       </c>
       <c r="G2199" t="n">
-        <v>436.49</v>
+        <v>4136.87</v>
       </c>
       <c r="H2199" t="n">
         <v>0</v>
@@ -75208,24 +75208,24 @@
     </row>
     <row r="2200">
       <c r="A2200" t="n">
-        <v>18162</v>
+        <v>18179</v>
       </c>
       <c r="B2200" s="2" t="n">
         <v>45988</v>
       </c>
       <c r="C2200" t="inlineStr">
         <is>
-          <t>Accounts Receivable</t>
+          <t>Cash at Bank</t>
         </is>
       </c>
       <c r="D2200" t="inlineStr">
         <is>
-          <t>Customer receipt</t>
+          <t>Supplier payment</t>
         </is>
       </c>
       <c r="E2200" t="inlineStr">
         <is>
-          <t>user_e</t>
+          <t>user_c</t>
         </is>
       </c>
       <c r="F2200" t="inlineStr">
@@ -75234,7 +75234,7 @@
         </is>
       </c>
       <c r="G2200" t="n">
-        <v>4136.87</v>
+        <v>4622.47</v>
       </c>
       <c r="H2200" t="n">
         <v>0</v>
@@ -75249,26 +75249,26 @@
       </c>
       <c r="C2201" t="inlineStr">
         <is>
-          <t>Cash at Bank</t>
+          <t>VAT Payable</t>
         </is>
       </c>
       <c r="D2201" t="inlineStr">
         <is>
-          <t>Supplier payment</t>
+          <t>Utility bill</t>
         </is>
       </c>
       <c r="E2201" t="inlineStr">
         <is>
-          <t>user_c</t>
+          <t>user_b</t>
         </is>
       </c>
       <c r="F2201" t="inlineStr">
         <is>
-          <t>manager_2</t>
+          <t>manager_1</t>
         </is>
       </c>
       <c r="G2201" t="n">
-        <v>4622.47</v>
+        <v>492.19</v>
       </c>
       <c r="H2201" t="n">
         <v>0</v>
@@ -75276,14 +75276,14 @@
     </row>
     <row r="2202">
       <c r="A2202" t="n">
-        <v>18181</v>
+        <v>18183</v>
       </c>
       <c r="B2202" s="2" t="n">
         <v>45988</v>
       </c>
       <c r="C2202" t="inlineStr">
         <is>
-          <t>VAT Payable</t>
+          <t>Cost of Sales</t>
         </is>
       </c>
       <c r="D2202" t="inlineStr">
@@ -75293,7 +75293,7 @@
       </c>
       <c r="E2202" t="inlineStr">
         <is>
-          <t>user_b</t>
+          <t>user_e</t>
         </is>
       </c>
       <c r="F2202" t="inlineStr">
@@ -75302,7 +75302,7 @@
         </is>
       </c>
       <c r="G2202" t="n">
-        <v>492.19</v>
+        <v>4849.87</v>
       </c>
       <c r="H2202" t="n">
         <v>0</v>
@@ -75310,7 +75310,7 @@
     </row>
     <row r="2203">
       <c r="A2203" t="n">
-        <v>18184</v>
+        <v>18187</v>
       </c>
       <c r="B2203" s="2" t="n">
         <v>45988</v>
@@ -75322,46 +75322,46 @@
       </c>
       <c r="D2203" t="inlineStr">
         <is>
-          <t>Utility bill</t>
+          <t>Supplier payment</t>
         </is>
       </c>
       <c r="E2203" t="inlineStr">
         <is>
-          <t>user_e</t>
+          <t>user_d</t>
         </is>
       </c>
       <c r="F2203" t="inlineStr">
         <is>
-          <t>manager_1</t>
+          <t>manager_2</t>
         </is>
       </c>
       <c r="G2203" t="n">
-        <v>4849.87</v>
+        <v>0</v>
       </c>
       <c r="H2203" t="n">
-        <v>0</v>
+        <v>4898.93</v>
       </c>
     </row>
     <row r="2204">
       <c r="A2204" t="n">
-        <v>18188</v>
+        <v>18199</v>
       </c>
       <c r="B2204" s="2" t="n">
         <v>45988</v>
       </c>
       <c r="C2204" t="inlineStr">
         <is>
-          <t>Cost of Sales</t>
+          <t>VAT Payable</t>
         </is>
       </c>
       <c r="D2204" t="inlineStr">
         <is>
-          <t>Supplier payment</t>
+          <t>Accrual</t>
         </is>
       </c>
       <c r="E2204" t="inlineStr">
         <is>
-          <t>user_d</t>
+          <t>user_c</t>
         </is>
       </c>
       <c r="F2204" t="inlineStr">
@@ -75370,10 +75370,10 @@
         </is>
       </c>
       <c r="G2204" t="n">
-        <v>0</v>
+        <v>48959.3</v>
       </c>
       <c r="H2204" t="n">
-        <v>4898.93</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2205">

</xml_diff>